<commit_message>
CZWN SWOB Excel/CSV: real date cells, wider columns, clean numbers
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012q8DP5dH322QPmsftUvE6c
</commit_message>
<xml_diff>
--- a/data/eccc/cfb-wainwright-czwn-swob-2026-10-17.xlsx
+++ b/data/eccc/cfb-wainwright-czwn-swob-2026-10-17.xlsx
@@ -17,7 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd hh:mm"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -55,13 +58,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,26 +435,26 @@
   <dimension ref="A1:Q21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="22.5" customWidth="1" min="2" max="2"/>
-    <col width="23.25" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="15.75" customWidth="1" min="7" max="7"/>
-    <col width="15.75" customWidth="1" min="8" max="8"/>
-    <col width="16.5" customWidth="1" min="9" max="9"/>
-    <col width="16.5" customWidth="1" min="10" max="10"/>
-    <col width="16.5" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12.75" customWidth="1" min="13" max="13"/>
-    <col width="12.75" customWidth="1" min="14" max="14"/>
-    <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="15" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="45" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>obs_time_utc</t>
@@ -537,20 +542,14 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-10-17 00:00</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-10-16 18:00</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2026-10-16 17:00</t>
-        </is>
+      <c r="A2" s="4" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>46311.75</v>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>46311.70833333334</v>
       </c>
       <c r="D2" t="n">
         <v>16.6</v>
@@ -579,19 +578,14 @@
       <c r="L2" t="n">
         <v>182</v>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-10-16 23:56</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>2026-10-16 17:56</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr"/>
+      <c r="M2" s="4" t="n">
+        <v>46311.99722222222</v>
+      </c>
+      <c r="N2" s="4" t="n">
+        <v>46311.74722222222</v>
+      </c>
       <c r="P2" t="n">
-        <v>93.28999999999999</v>
+        <v>93.29000000000001</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -600,20 +594,14 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-10-17 01:00</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-10-16 19:00</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2026-10-16 18:00</t>
-        </is>
+      <c r="A3" s="4" t="n">
+        <v>46312.04166666666</v>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>46311.79166666666</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>46311.75</v>
       </c>
       <c r="D3" t="n">
         <v>13.9</v>
@@ -642,19 +630,14 @@
       <c r="L3" t="n">
         <v>187</v>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-10-17 00:40</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>2026-10-16 18:40</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr"/>
+      <c r="M3" s="4" t="n">
+        <v>46312.02777777778</v>
+      </c>
+      <c r="N3" s="4" t="n">
+        <v>46311.77777777778</v>
+      </c>
       <c r="P3" t="n">
-        <v>93.22999999999999</v>
+        <v>93.23</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -663,20 +646,14 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-10-17 03:00</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-10-16 21:00</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2026-10-16 20:00</t>
-        </is>
+      <c r="A4" s="4" t="n">
+        <v>46312.125</v>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>46311.875</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>46311.83333333334</v>
       </c>
       <c r="D4" t="n">
         <v>10.7</v>
@@ -705,17 +682,12 @@
       <c r="L4" t="n">
         <v>194</v>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-10-17 02:49</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>2026-10-16 20:49</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr"/>
+      <c r="M4" s="4" t="n">
+        <v>46312.11736111111</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>46311.86736111111</v>
+      </c>
       <c r="P4" t="n">
         <v>93.12</v>
       </c>
@@ -726,20 +698,14 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-10-17 04:00</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-10-16 22:00</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2026-10-16 21:00</t>
-        </is>
+      <c r="A5" s="4" t="n">
+        <v>46312.16666666666</v>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>46311.91666666666</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>46311.875</v>
       </c>
       <c r="D5" t="n">
         <v>10</v>
@@ -768,17 +734,12 @@
       <c r="L5" t="n">
         <v>194</v>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-10-17 03:02</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>2026-10-16 21:02</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr"/>
+      <c r="M5" s="4" t="n">
+        <v>46312.12638888889</v>
+      </c>
+      <c r="N5" s="4" t="n">
+        <v>46311.87638888889</v>
+      </c>
       <c r="P5" t="n">
         <v>93.08</v>
       </c>
@@ -789,20 +750,14 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-10-17 05:00</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-10-16 23:00</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>2026-10-16 22:00</t>
-        </is>
+      <c r="A6" s="4" t="n">
+        <v>46312.20833333334</v>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>46311.95833333334</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>46311.91666666666</v>
       </c>
       <c r="D6" t="n">
         <v>8.699999999999999</v>
@@ -831,19 +786,14 @@
       <c r="L6" t="n">
         <v>206</v>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-10-17 04:04</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>2026-10-16 22:04</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr"/>
+      <c r="M6" s="4" t="n">
+        <v>46312.16944444444</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>46311.91944444444</v>
+      </c>
       <c r="P6" t="n">
-        <v>93.02000000000001</v>
+        <v>93.02</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -852,20 +802,14 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-10-17 06:00</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-10-17 00:00</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>2026-10-16 23:00</t>
-        </is>
+      <c r="A7" s="4" t="n">
+        <v>46312.25</v>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>46312</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>46311.95833333334</v>
       </c>
       <c r="D7" t="n">
         <v>8.1</v>
@@ -894,19 +838,14 @@
       <c r="L7" t="n">
         <v>143</v>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2026-10-17 05:58</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>2026-10-16 23:58</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr"/>
+      <c r="M7" s="4" t="n">
+        <v>46312.24861111111</v>
+      </c>
+      <c r="N7" s="4" t="n">
+        <v>46311.99861111111</v>
+      </c>
       <c r="P7" t="n">
-        <v>92.96000000000001</v>
+        <v>92.95999999999999</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -915,20 +854,14 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-10-17 07:00</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-10-17 01:00</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2026-10-17 00:00</t>
-        </is>
+      <c r="A8" s="4" t="n">
+        <v>46312.29166666666</v>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>46312.04166666666</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>46312</v>
       </c>
       <c r="D8" t="n">
         <v>6.6</v>
@@ -957,17 +890,12 @@
       <c r="L8" t="n">
         <v>160</v>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>2026-10-17 06:13</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>2026-10-17 00:13</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr"/>
+      <c r="M8" s="4" t="n">
+        <v>46312.25902777778</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>46312.00902777778</v>
+      </c>
       <c r="P8" t="n">
         <v>92.89</v>
       </c>
@@ -978,20 +906,14 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-10-17 08:00</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-10-17 02:00</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>2026-10-17 01:00</t>
-        </is>
+      <c r="A9" s="4" t="n">
+        <v>46312.33333333334</v>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>46312.08333333334</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>46312.04166666666</v>
       </c>
       <c r="D9" t="n">
         <v>5.7</v>
@@ -1020,17 +942,12 @@
       <c r="L9" t="n">
         <v>191</v>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>2026-10-17 07:13</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>2026-10-17 01:13</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr"/>
+      <c r="M9" s="4" t="n">
+        <v>46312.30069444444</v>
+      </c>
+      <c r="N9" s="4" t="n">
+        <v>46312.05069444444</v>
+      </c>
       <c r="P9" t="n">
         <v>92.83</v>
       </c>
@@ -1041,20 +958,14 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-10-17 09:00</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2026-10-17 03:00</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>2026-10-17 02:00</t>
-        </is>
+      <c r="A10" s="4" t="n">
+        <v>46312.375</v>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>46312.125</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>46312.08333333334</v>
       </c>
       <c r="D10" t="n">
         <v>7.1</v>
@@ -1083,17 +994,12 @@
       <c r="L10" t="n">
         <v>219</v>
       </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>2026-10-17 08:25</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>2026-10-17 02:25</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr"/>
+      <c r="M10" s="4" t="n">
+        <v>46312.35069444445</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>46312.10069444445</v>
+      </c>
       <c r="P10" t="n">
         <v>92.78</v>
       </c>
@@ -1104,20 +1010,14 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-10-17 11:00</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2026-10-17 05:00</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>2026-10-17 04:00</t>
-        </is>
+      <c r="A11" s="4" t="n">
+        <v>46312.45833333334</v>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>46312.20833333334</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>46312.16666666666</v>
       </c>
       <c r="D11" t="n">
         <v>6.6</v>
@@ -1146,17 +1046,12 @@
       <c r="L11" t="n">
         <v>199</v>
       </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>2026-10-17 10:59</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>2026-10-17 04:59</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr"/>
+      <c r="M11" s="4" t="n">
+        <v>46312.45763888889</v>
+      </c>
+      <c r="N11" s="4" t="n">
+        <v>46312.20763888889</v>
+      </c>
       <c r="P11" t="n">
         <v>92.58</v>
       </c>
@@ -1167,20 +1062,14 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-10-17 13:00</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2026-10-17 07:00</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>2026-10-17 06:00</t>
-        </is>
+      <c r="A12" s="4" t="n">
+        <v>46312.54166666666</v>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>46312.29166666666</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>46312.25</v>
       </c>
       <c r="D12" t="n">
         <v>6.7</v>
@@ -1209,19 +1098,14 @@
       <c r="L12" t="n">
         <v>220</v>
       </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>2026-10-17 12:05</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>2026-10-17 06:05</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr"/>
+      <c r="M12" s="4" t="n">
+        <v>46312.50347222222</v>
+      </c>
+      <c r="N12" s="4" t="n">
+        <v>46312.25347222222</v>
+      </c>
       <c r="P12" t="n">
-        <v>92.46000000000001</v>
+        <v>92.45999999999999</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1230,20 +1114,14 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-10-17 14:00</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>2026-10-17 08:00</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>2026-10-17 07:00</t>
-        </is>
+      <c r="A13" s="4" t="n">
+        <v>46312.58333333334</v>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>46312.33333333334</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>46312.29166666666</v>
       </c>
       <c r="D13" t="n">
         <v>6.1</v>
@@ -1272,17 +1150,12 @@
       <c r="L13" t="n">
         <v>218</v>
       </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>2026-10-17 13:06</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>2026-10-17 07:06</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr"/>
+      <c r="M13" s="4" t="n">
+        <v>46312.54583333333</v>
+      </c>
+      <c r="N13" s="4" t="n">
+        <v>46312.29583333333</v>
+      </c>
       <c r="P13" t="n">
         <v>92.34999999999999</v>
       </c>
@@ -1293,20 +1166,14 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-10-17 15:00</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>2026-10-17 09:00</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>2026-10-17 08:00</t>
-        </is>
+      <c r="A14" s="4" t="n">
+        <v>46312.625</v>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>46312.375</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>46312.33333333334</v>
       </c>
       <c r="D14" t="n">
         <v>7.6</v>
@@ -1335,17 +1202,12 @@
       <c r="L14" t="n">
         <v>220</v>
       </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>2026-10-17 14:58</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>2026-10-17 08:58</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr"/>
+      <c r="M14" s="4" t="n">
+        <v>46312.62361111111</v>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>46312.37361111111</v>
+      </c>
       <c r="P14" t="n">
         <v>92.25</v>
       </c>
@@ -1356,20 +1218,14 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-10-17 17:00</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>2026-10-17 11:00</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>2026-10-17 10:00</t>
-        </is>
+      <c r="A15" s="4" t="n">
+        <v>46312.70833333334</v>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>46312.45833333334</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>46312.41666666666</v>
       </c>
       <c r="D15" t="n">
         <v>13.9</v>
@@ -1398,17 +1254,12 @@
       <c r="L15" t="n">
         <v>202</v>
       </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>2026-10-17 16:52</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>2026-10-17 10:52</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr"/>
+      <c r="M15" s="4" t="n">
+        <v>46312.70277777778</v>
+      </c>
+      <c r="N15" s="4" t="n">
+        <v>46312.45277777778</v>
+      </c>
       <c r="P15" t="n">
         <v>92.06</v>
       </c>
@@ -1419,20 +1270,14 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-10-17 18:00</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>2026-10-17 12:00</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>2026-10-17 11:00</t>
-        </is>
+      <c r="A16" s="4" t="n">
+        <v>46312.75</v>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>46312.5</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>46312.45833333334</v>
       </c>
       <c r="D16" t="n">
         <v>15.2</v>
@@ -1461,17 +1306,12 @@
       <c r="L16" t="n">
         <v>200</v>
       </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>2026-10-17 17:01</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>2026-10-17 11:01</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr"/>
+      <c r="M16" s="4" t="n">
+        <v>46312.70902777778</v>
+      </c>
+      <c r="N16" s="4" t="n">
+        <v>46312.45902777778</v>
+      </c>
       <c r="P16" t="n">
         <v>92.01000000000001</v>
       </c>
@@ -1482,20 +1322,14 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-10-17 19:00</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>2026-10-17 13:00</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>2026-10-17 12:00</t>
-        </is>
+      <c r="A17" s="4" t="n">
+        <v>46312.79166666666</v>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>46312.54166666666</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>46312.5</v>
       </c>
       <c r="D17" t="n">
         <v>20.2</v>
@@ -1524,17 +1358,12 @@
       <c r="L17" t="n">
         <v>234</v>
       </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>2026-10-17 18:54</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>2026-10-17 12:54</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr"/>
+      <c r="M17" s="4" t="n">
+        <v>46312.7875</v>
+      </c>
+      <c r="N17" s="4" t="n">
+        <v>46312.5375</v>
+      </c>
       <c r="P17" t="n">
         <v>91.89</v>
       </c>
@@ -1545,20 +1374,14 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2026-10-17 20:00</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>2026-10-17 14:00</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>2026-10-17 13:00</t>
-        </is>
+      <c r="A18" s="4" t="n">
+        <v>46312.83333333334</v>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>46312.58333333334</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>46312.54166666666</v>
       </c>
       <c r="D18" t="n">
         <v>22.8</v>
@@ -1587,15 +1410,11 @@
       <c r="L18" t="n">
         <v>232</v>
       </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>2026-10-17 19:34</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>2026-10-17 13:34</t>
-        </is>
+      <c r="M18" s="4" t="n">
+        <v>46312.81527777778</v>
+      </c>
+      <c r="N18" s="4" t="n">
+        <v>46312.56527777778</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1603,7 +1422,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>91.82000000000001</v>
+        <v>91.81999999999999</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -1612,20 +1431,14 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2026-10-17 21:00</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>2026-10-17 15:00</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>2026-10-17 14:00</t>
-        </is>
+      <c r="A19" s="4" t="n">
+        <v>46312.875</v>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>46312.625</v>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>46312.58333333334</v>
       </c>
       <c r="D19" t="n">
         <v>23.3</v>
@@ -1654,15 +1467,11 @@
       <c r="L19" t="n">
         <v>246</v>
       </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>2026-10-17 20:48</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>2026-10-17 14:48</t>
-        </is>
+      <c r="M19" s="4" t="n">
+        <v>46312.86666666667</v>
+      </c>
+      <c r="N19" s="4" t="n">
+        <v>46312.61666666667</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1679,20 +1488,14 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-17 22:00</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-17 16:00</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-17 15:00</t>
-        </is>
+      <c r="A20" s="5" t="n">
+        <v>46312.91666666666</v>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>46312.66666666666</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>46312.625</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>12.9</v>
@@ -1721,15 +1524,11 @@
       <c r="L20" s="2" t="n">
         <v>269</v>
       </c>
-      <c r="M20" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-17 21:16</t>
-        </is>
-      </c>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-17 15:16</t>
-        </is>
+      <c r="M20" s="5" t="n">
+        <v>46312.88611111111</v>
+      </c>
+      <c r="N20" s="5" t="n">
+        <v>46312.63611111111</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1737,7 +1536,7 @@
         </is>
       </c>
       <c r="P20" s="2" t="n">
-        <v>92.27000000000001</v>
+        <v>92.27</v>
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
@@ -1746,20 +1545,14 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2026-10-17 23:00</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>2026-10-17 17:00</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>2026-10-17 16:00</t>
-        </is>
+      <c r="A21" s="4" t="n">
+        <v>46312.95833333334</v>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>46312.70833333334</v>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>46312.66666666666</v>
       </c>
       <c r="D21" t="n">
         <v>12</v>
@@ -1788,15 +1581,11 @@
       <c r="L21" t="n">
         <v>288</v>
       </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>2026-10-17 22:09</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>2026-10-17 16:09</t>
-        </is>
+      <c r="M21" s="4" t="n">
+        <v>46312.92291666667</v>
+      </c>
+      <c r="N21" s="4" t="n">
+        <v>46312.67291666667</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -1843,9 +1632,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -1888,9 +1675,7 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-    </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>

</xml_diff>